<commit_message>
criado coluna de controle se a RAT já foi lançado
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -1,270 +1,196 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HUSF" sheetId="1" r:id="rId1"/>
+    <sheet name="HUSF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
-  <si>
-    <t>PROJETO_ID</t>
-  </si>
-  <si>
-    <t>RAT_ID</t>
-  </si>
-  <si>
-    <t>DT_INICIO</t>
-  </si>
-  <si>
-    <t>DT_FIM</t>
-  </si>
-  <si>
-    <t>ATIVIDADE_ID</t>
-  </si>
-  <si>
-    <t>CLASSIFICACAO</t>
-  </si>
-  <si>
-    <t>DESCRICAO</t>
-  </si>
-  <si>
-    <t>MODALIDADE</t>
-  </si>
-  <si>
-    <t>Parametrização</t>
-  </si>
-  <si>
-    <t>Adicionar convênio no relatório 871</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>Verificar o caso que surgiu</t>
-  </si>
-  <si>
-    <t>Criar interação com o case da Philips (CS0528959 )</t>
-  </si>
-  <si>
-    <t>Aconteceu uma situação com um KIT aonde não gerou os horários. Lote: 1819946</t>
-  </si>
-  <si>
-    <t>Realizar teste na procedure para considerar kits</t>
-  </si>
-  <si>
-    <t>Call com cassiana para analisar devolução que foi realizado com prescrições distintas</t>
-  </si>
-  <si>
-    <t>Analisar caso de erro</t>
-  </si>
-  <si>
-    <t>Adicionar na procedure um log. Criado versão nova do script.</t>
-  </si>
-  <si>
-    <t>Assistir vídeo da conexão realizada pela Cassiana a respeito do problema do histórico do lote</t>
-  </si>
-  <si>
-    <t>Realizado Call com Cassiana aonde ela demonstrou problema no setor do lote</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="180" formatCode="dd/mm/yyyy\ hh:mm;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="6">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm;@"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ h:mm"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
-    <font>
+  <fonts count="22">
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF333333"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="CentraleSansCndBook"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <u/>
+      <color rgb="FF333333"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="CentraleSansCnd"/>
+      <charset val="134"/>
+      <color rgb="FF333333"/>
+      <sz val="10.45"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
+      <color rgb="FF800080"/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <color rgb="FFFF0000"/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color rgb="FF3F3F76"/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <color rgb="FF006100"/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color rgb="FF9C0006"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -564,165 +490,175 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -970,7 +906,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -979,7 +915,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -992,11 +928,74 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1248,313 +1247,590 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelCol="7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.142857142857141" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="11.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="15.5714285714286" customWidth="1"/>
-    <col min="4" max="4" width="16.5714285714286" customWidth="1"/>
-    <col min="5" max="5" width="12.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="18.2857142857143" customWidth="1"/>
-    <col min="7" max="7" width="56.2857142857143" customWidth="1"/>
+    <col width="11.1428571428571" customWidth="1" style="1" min="1" max="1"/>
+    <col width="15.5714285714286" customWidth="1" style="1" min="3" max="3"/>
+    <col width="16.5714285714286" customWidth="1" style="1" min="4" max="4"/>
+    <col width="12.5714285714286" customWidth="1" style="1" min="5" max="5"/>
+    <col width="18.2857142857143" customWidth="1" style="1" min="6" max="6"/>
+    <col width="56.2857142857143" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12.2857142857143" customWidth="1" style="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>PROJETO_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>RAT_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>DT_INICIO</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>DT_FIM</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>ATIVIDADE_ID</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>CLASSIFICACAO</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>DESCRICAO</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>MODALIDADE</t>
+        </is>
+      </c>
+      <c r="I1" s="0" t="inlineStr">
+        <is>
+          <t>LANCADA</t>
+        </is>
       </c>
     </row>
-    <row r="2" ht="15" spans="1:8">
-      <c r="A2">
+    <row r="2" ht="15" customHeight="1" s="1">
+      <c r="A2" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C2" s="1">
-        <v>46154.6458333333</v>
-      </c>
-      <c r="D2" s="1">
-        <v>46154.6541666667</v>
-      </c>
-      <c r="E2">
+      <c r="C2" s="6" t="n">
+        <v>46154.64583333334</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>46154.65416666667</v>
+      </c>
+      <c r="E2" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" t="s">
-        <v>10</v>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>Adicionar convênio no relatório 871</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I2" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="15" spans="1:8">
-      <c r="A3">
+    <row r="3" ht="15" customHeight="1" s="1">
+      <c r="A3" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C3" s="1">
-        <v>46155.2430555556</v>
-      </c>
-      <c r="D3" s="1">
-        <v>46155.3486111111</v>
-      </c>
-      <c r="E3">
+      <c r="C3" s="6" t="n">
+        <v>46155.24305555555</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>46155.34861111111</v>
+      </c>
+      <c r="E3" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" t="s">
-        <v>10</v>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Verificar o caso que surgiu</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="4" ht="15" spans="1:8">
-      <c r="A4">
+    <row r="4" ht="15" customHeight="1" s="1">
+      <c r="A4" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="6" t="n">
         <v>46155.3625</v>
       </c>
-      <c r="D4" s="1">
-        <v>46155.3659722222</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="6" t="n">
+        <v>46155.36597222222</v>
+      </c>
+      <c r="E4" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>10</v>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Criar interação com o case da Philips (CS0528959 )</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I4" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="15" spans="1:8">
-      <c r="A5">
+    <row r="5" ht="15" customHeight="1" s="1">
+      <c r="A5" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C5" s="1">
-        <v>46157.5486111111</v>
-      </c>
-      <c r="D5" s="1">
-        <v>46157.5652777778</v>
-      </c>
-      <c r="E5">
+      <c r="C5" s="6" t="n">
+        <v>46157.54861111111</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>46157.56527777778</v>
+      </c>
+      <c r="E5" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s">
-        <v>10</v>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>Aconteceu uma situação com um KIT aonde não gerou os horários. Lote: 1819946</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="15" spans="1:8">
-      <c r="A6">
+    <row r="6" ht="15" customHeight="1" s="1">
+      <c r="A6" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C6" s="1">
-        <v>46160.3229166667</v>
-      </c>
-      <c r="D6" s="1">
-        <v>46160.3666666667</v>
-      </c>
-      <c r="E6">
+      <c r="C6" s="6" t="n">
+        <v>46160.32291666666</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>46160.36666666667</v>
+      </c>
+      <c r="E6" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" t="s">
-        <v>10</v>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Realizar teste na procedure para considerar kits</t>
+        </is>
+      </c>
+      <c r="H6" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="7" ht="15" spans="1:8">
-      <c r="A7">
+    <row r="7" ht="15" customHeight="1" s="1">
+      <c r="A7" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C7" s="1">
-        <v>46160.6777777778</v>
-      </c>
-      <c r="D7" s="1">
-        <v>46160.6944444444</v>
-      </c>
-      <c r="E7">
+      <c r="C7" s="6" t="n">
+        <v>46160.67777777778</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>46160.69444444445</v>
+      </c>
+      <c r="E7" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>10</v>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Call com cassiana para analisar devolução que foi realizado com prescrições distintas</t>
+        </is>
+      </c>
+      <c r="H7" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="8" ht="15" spans="1:8">
-      <c r="A8">
+    <row r="8" ht="15" customHeight="1" s="1">
+      <c r="A8" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C8" s="1">
-        <v>46161.5347222222</v>
-      </c>
-      <c r="D8" s="1">
-        <v>46161.5833333333</v>
-      </c>
-      <c r="E8">
+      <c r="C8" s="6" t="n">
+        <v>46161.53472222222</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>46161.58333333334</v>
+      </c>
+      <c r="E8" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" t="s">
-        <v>10</v>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>Analisar caso de erro</t>
+        </is>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="9" ht="15" spans="1:8">
-      <c r="A9">
+    <row r="9" ht="15" customHeight="1" s="1">
+      <c r="A9" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C9" s="1">
-        <v>46162.2708333333</v>
-      </c>
-      <c r="D9" s="1">
+      <c r="C9" s="6" t="n">
+        <v>46162.27083333334</v>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>46162.3125</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" t="s">
-        <v>10</v>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Adicionar na procedure um log. Criado versão nova do script.</t>
+        </is>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="10" ht="15" spans="1:8">
-      <c r="A10">
+    <row r="10" ht="15" customHeight="1" s="1">
+      <c r="A10" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C10" s="1">
-        <v>46162.3472222222</v>
-      </c>
-      <c r="D10" s="1">
-        <v>46162.4041666667</v>
-      </c>
-      <c r="E10">
+      <c r="C10" s="6" t="n">
+        <v>46162.34722222222</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>46162.40416666667</v>
+      </c>
+      <c r="E10" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" t="s">
-        <v>10</v>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Assistir vídeo da conexão realizada pela Cassiana a respeito do problema do histórico do lote</t>
+        </is>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="11" ht="15" spans="1:8">
-      <c r="A11">
+    <row r="11" ht="15" customHeight="1" s="1">
+      <c r="A11" s="0" t="n">
         <v>694</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="0" t="n">
         <v>31873</v>
       </c>
-      <c r="C11" s="1">
-        <v>46162.7083333333</v>
-      </c>
-      <c r="D11" s="1">
-        <v>46162.7166666667</v>
-      </c>
-      <c r="E11">
+      <c r="C11" s="6" t="n">
+        <v>46162.70833333334</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>46162.71666666667</v>
+      </c>
+      <c r="E11" s="0" t="n">
         <v>30631</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G11" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" t="s">
-        <v>10</v>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>Realizado Call com Cassiana aonde ela demonstrou problema no setor do lote</t>
+        </is>
+      </c>
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
-    <row r="13" spans="1:8">
-      <c r="D13" s="3" t="s">
-        <v>20</v>
+    <row r="12" ht="15" customHeight="1" s="1">
+      <c r="A12" s="0" t="n">
+        <v>694</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>31908</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>46167.375</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>46167.41597222222</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <v>30631</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>Call com Cassiana aonde foi demonstrado o cenário aonde não houve a movimentação do paciente para fora do CC, e outra aonde identificamos um erro na procedure.  Esta será corrigida.</t>
+        </is>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I12" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="1">
+      <c r="A13" s="0" t="n">
+        <v>694</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>31908</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>46167.41666666666</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>46167.46388888889</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <v>30631</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>Correção na Procedure</t>
+        </is>
+      </c>
+      <c r="H13" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="1">
+      <c r="A14" s="0" t="n">
+        <v>694</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>31908</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>46167.47916666666</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>46167.58958333333</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <v>30631</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>Correção na Procedure</t>
+        </is>
+      </c>
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="1">
+      <c r="A15" s="0" t="n">
+        <v>694</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>31908</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>46167.73611111111</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>46167.75</v>
+      </c>
+      <c r="E15" s="0" t="n">
+        <v>30631</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Parametrização</t>
+        </is>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>Analisa de devolução passada e identificado erro na procedure, esta foi corrigida</t>
+        </is>
+      </c>
+      <c r="H15" s="0" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="256" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" paperSize="256"/>
 </worksheet>
 </file>
</xml_diff>